<commit_message>
Workbook hardened and documents aligned: gap rule, blank-input rule, false-consensus guard, trip-wire not-measured text; parity fixtures added
</commit_message>
<xml_diff>
--- a/docs/benchmarks/PerformanceVP-Diagnostic-Workbook.xlsx
+++ b/docs/benchmarks/PerformanceVP-Diagnostic-Workbook.xlsx
@@ -3090,7 +3090,7 @@
         <v>2.66666666666667</v>
       </c>
       <c r="P5" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K5),B32*((1+L5*O5/M5)^N5-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K5),ISNUMBER(B32)),B32*((1+L5*O5/M5)^N5-1),"")</f>
         <v>0.322379936001943</v>
       </c>
       <c r="Q5" s="15" t="n">
@@ -3098,7 +3098,7 @@
         <v>0.24410008424858</v>
       </c>
       <c r="R5" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K5),P5*Q5,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K5),ISNUMBER(P5)),P5*Q5,"")</f>
         <v>0.0786929695381262</v>
       </c>
       <c r="S5" s="6" t="n">
@@ -3160,7 +3160,7 @@
         <v>3.36171428571429</v>
       </c>
       <c r="P6" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K6),B32*((1+L6*O6/M6)^N6-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K6),ISNUMBER(B32)),B32*((1+L6*O6/M6)^N6-1),"")</f>
         <v>0.174504621207843</v>
       </c>
       <c r="Q6" s="15" t="n">
@@ -3168,7 +3168,7 @@
         <v>0.301381589646565</v>
       </c>
       <c r="R6" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K6),P6*Q6,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K6),ISNUMBER(P6)),P6*Q6,"")</f>
         <v>0.0525924801402914</v>
       </c>
       <c r="S6" s="6" t="n">
@@ -3230,7 +3230,7 @@
         <v>5.55</v>
       </c>
       <c r="P7" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K7),B32*((1+L7*O7/M7)^N7-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K7),ISNUMBER(B32)),B32*((1+L7*O7/M7)^N7-1),"")</f>
         <v>0.38310353465438</v>
       </c>
       <c r="Q7" s="15" t="n">
@@ -3238,7 +3238,7 @@
         <v>0.517757086577807</v>
       </c>
       <c r="R7" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K7),P7*Q7,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K7),ISNUMBER(P7)),P7*Q7,"")</f>
         <v>0.198354569960312</v>
       </c>
       <c r="S7" s="6" t="n">
@@ -3300,7 +3300,7 @@
         <v>4.4025</v>
       </c>
       <c r="P8" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K8),B32*((1+L8*O8/M8)^N8-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K8),ISNUMBER(B32)),B32*((1+L8*O8/M8)^N8-1),"")</f>
         <v>0.304201818304714</v>
       </c>
       <c r="Q8" s="15" t="n">
@@ -3308,7 +3308,7 @@
         <v>0.39961566292604</v>
       </c>
       <c r="R8" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K8),P8*Q8,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K8),ISNUMBER(P8)),P8*Q8,"")</f>
         <v>0.121563811285145</v>
       </c>
       <c r="S8" s="6" t="n">
@@ -3370,7 +3370,7 @@
         <v>1.8</v>
       </c>
       <c r="P9" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K9),B32*((1+L9*O9/M9)^N9-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K9),ISNUMBER(B32)),B32*((1+L9*O9/M9)^N9-1),"")</f>
         <v>0.06238099439244</v>
       </c>
       <c r="Q9" s="15" t="n">
@@ -3378,7 +3378,7 @@
         <v>0.183705424332345</v>
       </c>
       <c r="R9" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K9),P9*Q9,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K9),ISNUMBER(P9)),P9*Q9,"")</f>
         <v>0.0114597270451368</v>
       </c>
       <c r="S9" s="6" t="n">
@@ -3440,7 +3440,7 @@
         <v>3.9</v>
       </c>
       <c r="P10" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K10),B32*((1+L10*O10/M10)^N10-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K10),ISNUMBER(B32)),B32*((1+L10*O10/M10)^N10-1),"")</f>
         <v>0.79858225849194</v>
       </c>
       <c r="Q10" s="15" t="n">
@@ -3448,7 +3448,7 @@
         <v>0.350591147358275</v>
       </c>
       <c r="R10" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K10),P10*Q10,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K10),ISNUMBER(P10)),P10*Q10,"")</f>
         <v>0.279975870264652</v>
       </c>
       <c r="S10" s="6" t="n">
@@ -3495,7 +3495,7 @@
         <v>3</v>
       </c>
       <c r="P11" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K11),B32*((1+L11*O11/M11)^N11-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K11),ISNUMBER(B32)),B32*((1+L11*O11/M11)^N11-1),"")</f>
         <v>0.247122761890417</v>
       </c>
       <c r="Q11" s="15" t="n">
@@ -3503,7 +3503,7 @@
         <v>0.270627395273177</v>
       </c>
       <c r="R11" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K11),P11*Q11,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K11),ISNUMBER(P11)),P11*Q11,"")</f>
         <v>0.066878189363117</v>
       </c>
       <c r="S11" s="6" t="n">
@@ -3565,7 +3565,7 @@
         <v>5.4</v>
       </c>
       <c r="P12" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K12),B32*((1+L12*O12/M12)^N12-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K12),ISNUMBER(B32)),B32*((1+L12*O12/M12)^N12-1),"")</f>
         <v>0.333318116897318</v>
       </c>
       <c r="Q12" s="15" t="n">
@@ -3573,7 +3573,7 @@
         <v>0.502139544587047</v>
       </c>
       <c r="R12" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K12),P12*Q12,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K12),ISNUMBER(P12)),P12*Q12,"")</f>
         <v>0.167372207421431</v>
       </c>
       <c r="S12" s="6" t="n">
@@ -3635,7 +3635,7 @@
         <v>7.5</v>
       </c>
       <c r="P13" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K13),B32*((1+L13*O13/M13)^N13-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K13),ISNUMBER(B32)),B32*((1+L13*O13/M13)^N13-1),"")</f>
         <v>0.462324251799247</v>
       </c>
       <c r="Q13" s="15" t="n">
@@ -3643,7 +3643,7 @@
         <v>0.707559030880924</v>
       </c>
       <c r="R13" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K13),P13*Q13,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K13),ISNUMBER(P13)),P13*Q13,"")</f>
         <v>0.327121699555823</v>
       </c>
       <c r="S13" s="6" t="n">
@@ -3705,7 +3705,7 @@
         <v>7.1315625</v>
       </c>
       <c r="P14" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K14),B32*((1+L14*O14/M14)^N14-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K14),ISNUMBER(B32)),B32*((1+L14*O14/M14)^N14-1),"")</f>
         <v>0.62206329873543</v>
       </c>
       <c r="Q14" s="15" t="n">
@@ -3713,7 +3713,7 @@
         <v>0.674814622014799</v>
       </c>
       <c r="R14" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K14),P14*Q14,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K14),ISNUMBER(P14)),P14*Q14,"")</f>
         <v>0.419777409805429</v>
       </c>
       <c r="S14" s="6" t="n">
@@ -3775,7 +3775,7 @@
         <v>4.725</v>
       </c>
       <c r="P15" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K15),B32*((1+L15*O15/M15)^N15-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K15),ISNUMBER(B32)),B32*((1+L15*O15/M15)^N15-1),"")</f>
         <v>0.345429724605946</v>
       </c>
       <c r="Q15" s="15" t="n">
@@ -3783,7 +3783,7 @@
         <v>0.432246389288702</v>
       </c>
       <c r="R15" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K15),P15*Q15,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K15),ISNUMBER(P15)),P15*Q15,"")</f>
         <v>0.149310751213911</v>
       </c>
       <c r="S15" s="6" t="n">
@@ -3830,7 +3830,7 @@
         <v>8.925</v>
       </c>
       <c r="P16" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K16),B32*((1+L16*O16/M16)^N16-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K16),ISNUMBER(B32)),B32*((1+L16*O16/M16)^N16-1),"")</f>
         <v>0.520096817490926</v>
       </c>
       <c r="Q16" s="15" t="n">
@@ -3838,7 +3838,7 @@
         <v>0.81416566052437</v>
       </c>
       <c r="R16" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K16),P16*Q16,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K16),ISNUMBER(P16)),P16*Q16,"")</f>
         <v>0.423444968949122</v>
       </c>
       <c r="S16" s="6" t="n">
@@ -3900,7 +3900,7 @@
         <v>11.25</v>
       </c>
       <c r="P17" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K17),B32*((1+L17*O17/M17)^N17-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K17),ISNUMBER(B32)),B32*((1+L17*O17/M17)^N17-1),"")</f>
         <v>0.329092109761143</v>
       </c>
       <c r="Q17" s="15" t="n">
@@ -3908,7 +3908,7 @@
         <v>0.920272718567815</v>
       </c>
       <c r="R17" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K17),P17*Q17,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K17),ISNUMBER(P17)),P17*Q17,"")</f>
         <v>0.302854490509105</v>
       </c>
       <c r="S17" s="6" t="n">
@@ -3970,7 +3970,7 @@
         <v>5.7</v>
       </c>
       <c r="P18" s="18" t="n">
-        <f aca="false">IF(ISNUMBER(K18),B32*((1+L18*O18/M18)^N18-1),"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K18),ISNUMBER(B32)),B32*((1+L18*O18/M18)^N18-1),"")</f>
         <v>0.250517705812853</v>
       </c>
       <c r="Q18" s="15" t="n">
@@ -3978,7 +3978,7 @@
         <v>0.533340012997247</v>
       </c>
       <c r="R18" s="15" t="n">
-        <f aca="false">IF(ISNUMBER(K18),P18*Q18,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(K18),ISNUMBER(P18)),P18*Q18,"")</f>
         <v>0.133611116474268</v>
       </c>
       <c r="S18" s="6" t="n">
@@ -4459,7 +4459,7 @@
         <v>432</v>
       </c>
       <c r="B51" s="29" t="str">
-        <f aca="false">IF(MIN(IF('Tier Assignment'!$E$5="Low",1,IF('Tier Assignment'!$E$5="Medium",2,3)),IF('Tier Assignment'!$E$6="Low",1,IF('Tier Assignment'!$E$6="Medium",2,3)),IF('Tier Assignment'!$E$7="Low",1,IF('Tier Assignment'!$E$7="Medium",2,3)),IF('Tier Assignment'!$E$8="Low",1,IF('Tier Assignment'!$E$8="Medium",2,3)),IF('Tier Assignment'!$E$9="Low",1,IF('Tier Assignment'!$E$9="Medium",2,3)),IF('Tier Assignment'!$E$10="Low",1,IF('Tier Assignment'!$E$10="Medium",2,3)),IF('Tier Assignment'!$E$11="Low",1,IF('Tier Assignment'!$E$11="Medium",2,3)),IF('Tier Assignment'!$E$12="Low",1,IF('Tier Assignment'!$E$12="Medium",2,3)),IF('Tier Assignment'!$E$13="Low",1,IF('Tier Assignment'!$E$13="Medium",2,3)),IF('Tier Assignment'!$E$17="Low",1,IF('Tier Assignment'!$E$17="Medium",2,3)),IF('Tier Assignment'!$E$18="Low",1,IF('Tier Assignment'!$E$18="Medium",2,3)),IF('Tier Assignment'!$E$19="Low",1,IF('Tier Assignment'!$E$19="Medium",2,3)),IF('Tier Assignment'!$E$20="Low",1,IF('Tier Assignment'!$E$20="Medium",2,3)),IF('Tier Assignment'!$E$21="Low",1,IF('Tier Assignment'!$E$21="Medium",2,3)),IF('Tier Assignment'!$E$22="Low",1,IF('Tier Assignment'!$E$22="Medium",2,3)),IF('Tier Assignment'!$E$23="Low",1,IF('Tier Assignment'!$E$23="Medium",2,3)),IF('Tier Assignment'!$E$24="Low",1,IF('Tier Assignment'!$E$24="Medium",2,3)))=1,"Low",IF(MIN(IF('Tier Assignment'!$E$5="Low",1,IF('Tier Assignment'!$E$5="Medium",2,3)),IF('Tier Assignment'!$E$6="Low",1,IF('Tier Assignment'!$E$6="Medium",2,3)),IF('Tier Assignment'!$E$7="Low",1,IF('Tier Assignment'!$E$7="Medium",2,3)),IF('Tier Assignment'!$E$8="Low",1,IF('Tier Assignment'!$E$8="Medium",2,3)),IF('Tier Assignment'!$E$9="Low",1,IF('Tier Assignment'!$E$9="Medium",2,3)),IF('Tier Assignment'!$E$10="Low",1,IF('Tier Assignment'!$E$10="Medium",2,3)),IF('Tier Assignment'!$E$11="Low",1,IF('Tier Assignment'!$E$11="Medium",2,3)),IF('Tier Assignment'!$E$12="Low",1,IF('Tier Assignment'!$E$12="Medium",2,3)),IF('Tier Assignment'!$E$13="Low",1,IF('Tier Assignment'!$E$13="Medium",2,3)),IF('Tier Assignment'!$E$17="Low",1,IF('Tier Assignment'!$E$17="Medium",2,3)),IF('Tier Assignment'!$E$18="Low",1,IF('Tier Assignment'!$E$18="Medium",2,3)),IF('Tier Assignment'!$E$19="Low",1,IF('Tier Assignment'!$E$19="Medium",2,3)),IF('Tier Assignment'!$E$20="Low",1,IF('Tier Assignment'!$E$20="Medium",2,3)),IF('Tier Assignment'!$E$21="Low",1,IF('Tier Assignment'!$E$21="Medium",2,3)),IF('Tier Assignment'!$E$22="Low",1,IF('Tier Assignment'!$E$22="Medium",2,3)),IF('Tier Assignment'!$E$23="Low",1,IF('Tier Assignment'!$E$23="Medium",2,3)),IF('Tier Assignment'!$E$24="Low",1,IF('Tier Assignment'!$E$24="Medium",2,3)))=2,"Medium","High"))</f>
+        <f aca="false">IF(ISNUMBER(B32),IF(MIN(IF('Tier Assignment'!$E$5="Low",1,IF('Tier Assignment'!$E$5="Medium",2,3)),IF('Tier Assignment'!$E$6="Low",1,IF('Tier Assignment'!$E$6="Medium",2,3)),IF('Tier Assignment'!$E$7="Low",1,IF('Tier Assignment'!$E$7="Medium",2,3)),IF('Tier Assignment'!$E$8="Low",1,IF('Tier Assignment'!$E$8="Medium",2,3)),IF('Tier Assignment'!$E$9="Low",1,IF('Tier Assignment'!$E$9="Medium",2,3)),IF('Tier Assignment'!$E$10="Low",1,IF('Tier Assignment'!$E$10="Medium",2,3)),IF('Tier Assignment'!$E$11="Low",1,IF('Tier Assignment'!$E$11="Medium",2,3)),IF('Tier Assignment'!$E$12="Low",1,IF('Tier Assignment'!$E$12="Medium",2,3)),IF('Tier Assignment'!$E$13="Low",1,IF('Tier Assignment'!$E$13="Medium",2,3)),IF('Tier Assignment'!$E$17="Low",1,IF('Tier Assignment'!$E$17="Medium",2,3)),IF('Tier Assignment'!$E$18="Low",1,IF('Tier Assignment'!$E$18="Medium",2,3)),IF('Tier Assignment'!$E$19="Low",1,IF('Tier Assignment'!$E$19="Medium",2,3)),IF('Tier Assignment'!$E$20="Low",1,IF('Tier Assignment'!$E$20="Medium",2,3)),IF('Tier Assignment'!$E$21="Low",1,IF('Tier Assignment'!$E$21="Medium",2,3)),IF('Tier Assignment'!$E$22="Low",1,IF('Tier Assignment'!$E$22="Medium",2,3)),IF('Tier Assignment'!$E$23="Low",1,IF('Tier Assignment'!$E$23="Medium",2,3)),IF('Tier Assignment'!$E$24="Low",1,IF('Tier Assignment'!$E$24="Medium",2,3)))=1,"Low",IF(MIN(IF('Tier Assignment'!$E$5="Low",1,IF('Tier Assignment'!$E$5="Medium",2,3)),IF('Tier Assignment'!$E$6="Low",1,IF('Tier Assignment'!$E$6="Medium",2,3)),IF('Tier Assignment'!$E$7="Low",1,IF('Tier Assignment'!$E$7="Medium",2,3)),IF('Tier Assignment'!$E$8="Low",1,IF('Tier Assignment'!$E$8="Medium",2,3)),IF('Tier Assignment'!$E$9="Low",1,IF('Tier Assignment'!$E$9="Medium",2,3)),IF('Tier Assignment'!$E$10="Low",1,IF('Tier Assignment'!$E$10="Medium",2,3)),IF('Tier Assignment'!$E$11="Low",1,IF('Tier Assignment'!$E$11="Medium",2,3)),IF('Tier Assignment'!$E$12="Low",1,IF('Tier Assignment'!$E$12="Medium",2,3)),IF('Tier Assignment'!$E$13="Low",1,IF('Tier Assignment'!$E$13="Medium",2,3)),IF('Tier Assignment'!$E$17="Low",1,IF('Tier Assignment'!$E$17="Medium",2,3)),IF('Tier Assignment'!$E$18="Low",1,IF('Tier Assignment'!$E$18="Medium",2,3)),IF('Tier Assignment'!$E$19="Low",1,IF('Tier Assignment'!$E$19="Medium",2,3)),IF('Tier Assignment'!$E$20="Low",1,IF('Tier Assignment'!$E$20="Medium",2,3)),IF('Tier Assignment'!$E$21="Low",1,IF('Tier Assignment'!$E$21="Medium",2,3)),IF('Tier Assignment'!$E$22="Low",1,IF('Tier Assignment'!$E$22="Medium",2,3)),IF('Tier Assignment'!$E$23="Low",1,IF('Tier Assignment'!$E$23="Medium",2,3)),IF('Tier Assignment'!$E$24="Low",1,IF('Tier Assignment'!$E$24="Medium",2,3)))=2,"Medium","High")),"")</f>
         <v>High</v>
       </c>
     </row>
@@ -4707,7 +4707,7 @@
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="27" t="str">
-        <f aca="false">IF((IF('Motivation Inputs'!D52&lt;&gt;"","Pay equity trip-wire breached; ","")&amp;IF('Motivation Inputs'!D53&lt;&gt;"","Fairness trip-wire breached; ","")&amp;IF('Motivation Inputs'!D54&lt;&gt;"","Basic conditions trip-wire breached; ","")&amp;IF(AND(ISNUMBER(DLP!B52),DLP!B52&lt;50),"Decision latency critical (overall DLS below 50); ",""))="","No critical findings identified",LEFT((IF('Motivation Inputs'!D52&lt;&gt;"","Pay equity trip-wire breached; ","")&amp;IF('Motivation Inputs'!D53&lt;&gt;"","Fairness trip-wire breached; ","")&amp;IF('Motivation Inputs'!D54&lt;&gt;"","Basic conditions trip-wire breached; ","")&amp;IF(AND(ISNUMBER(DLP!B52),DLP!B52&lt;50),"Decision latency critical (overall DLS below 50); ","")),LEN((IF('Motivation Inputs'!D52&lt;&gt;"","Pay equity trip-wire breached; ","")&amp;IF('Motivation Inputs'!D53&lt;&gt;"","Fairness trip-wire breached; ","")&amp;IF('Motivation Inputs'!D54&lt;&gt;"","Basic conditions trip-wire breached; ","")&amp;IF(AND(ISNUMBER(DLP!B52),DLP!B52&lt;50),"Decision latency critical (overall DLS below 50); ","")))-2))</f>
+        <f aca="false">IF((IF('Motivation Inputs'!D52&lt;&gt;"","Pay equity trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C52)),"Pay equity trip-wire not measured; ",""))&amp;IF('Motivation Inputs'!D53&lt;&gt;"","Fairness trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C53)),"Fairness trip-wire not measured; ",""))&amp;IF('Motivation Inputs'!D54&lt;&gt;"","Basic conditions trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C54)),"Basic conditions trip-wire not measured; ",""))&amp;IF(AND(ISNUMBER(DLP!B52),DLP!B52&lt;50),"Decision latency critical (overall DLS below 50); ",""))="","No critical findings identified",LEFT((IF('Motivation Inputs'!D52&lt;&gt;"","Pay equity trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C52)),"Pay equity trip-wire not measured; ",""))&amp;IF('Motivation Inputs'!D53&lt;&gt;"","Fairness trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C53)),"Fairness trip-wire not measured; ",""))&amp;IF('Motivation Inputs'!D54&lt;&gt;"","Basic conditions trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C54)),"Basic conditions trip-wire not measured; ",""))&amp;IF(AND(ISNUMBER(DLP!B52),DLP!B52&lt;50),"Decision latency critical (overall DLS below 50); ","")),LEN((IF('Motivation Inputs'!D52&lt;&gt;"","Pay equity trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C52)),"Pay equity trip-wire not measured; ",""))&amp;IF('Motivation Inputs'!D53&lt;&gt;"","Fairness trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C53)),"Fairness trip-wire not measured; ",""))&amp;IF('Motivation Inputs'!D54&lt;&gt;"","Basic conditions trip-wire breached; ",IF(NOT(ISNUMBER('Motivation Inputs'!C54)),"Basic conditions trip-wire not measured; ",""))&amp;IF(AND(ISNUMBER(DLP!B52),DLP!B52&lt;50),"Decision latency critical (overall DLS below 50); ","")))-2))</f>
         <v>Basic conditions trip-wire breached</v>
       </c>
     </row>
@@ -4731,7 +4731,7 @@
         <v>47</v>
       </c>
       <c r="C29" s="33" t="n">
-        <f aca="false">'Capability Inputs'!B52</f>
+        <f aca="false">IF('Capability Inputs'!B52="","",'Capability Inputs'!B52)</f>
         <v>0.78</v>
       </c>
     </row>
@@ -4740,7 +4740,7 @@
         <v>53</v>
       </c>
       <c r="C30" s="33" t="n">
-        <f aca="false">'Motivation Inputs'!B16</f>
+        <f aca="false">IF('Motivation Inputs'!B16="","",'Motivation Inputs'!B16)</f>
         <v>0.78</v>
       </c>
     </row>
@@ -4749,7 +4749,7 @@
         <v>55</v>
       </c>
       <c r="C31" s="33" t="n">
-        <f aca="false">'Motivation Inputs'!B28</f>
+        <f aca="false">IF('Motivation Inputs'!B28="","",'Motivation Inputs'!B28)</f>
         <v>0.78</v>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
         <v>57</v>
       </c>
       <c r="C32" s="33" t="n">
-        <f aca="false">'Motivation Inputs'!B38</f>
+        <f aca="false">IF('Motivation Inputs'!B38="","",'Motivation Inputs'!B38)</f>
         <v>0.76</v>
       </c>
     </row>
@@ -4767,7 +4767,7 @@
         <v>59</v>
       </c>
       <c r="C33" s="33" t="n">
-        <f aca="false">'Motivation Inputs'!B47</f>
+        <f aca="false">IF('Motivation Inputs'!B47="","",'Motivation Inputs'!B47)</f>
         <v>0.76</v>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
         <v>66</v>
       </c>
       <c r="C34" s="33" t="n">
-        <f aca="false">'Opportunity Inputs'!B19</f>
+        <f aca="false">IF('Opportunity Inputs'!B19="","",'Opportunity Inputs'!B19)</f>
         <v>0.8</v>
       </c>
     </row>
@@ -4785,7 +4785,7 @@
         <v>69</v>
       </c>
       <c r="C35" s="33" t="n">
-        <f aca="false">'Opportunity Inputs'!B36</f>
+        <f aca="false">IF('Opportunity Inputs'!B36="","",'Opportunity Inputs'!B36)</f>
         <v>0.82</v>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
         <v>71</v>
       </c>
       <c r="C36" s="33" t="n">
-        <f aca="false">'Opportunity Inputs'!B52</f>
+        <f aca="false">IF('Opportunity Inputs'!B52="","",'Opportunity Inputs'!B52)</f>
         <v>0.83</v>
       </c>
     </row>
@@ -4803,7 +4803,7 @@
         <v>73</v>
       </c>
       <c r="C37" s="33" t="n">
-        <f aca="false">'Opportunity Inputs'!B65</f>
+        <f aca="false">IF('Opportunity Inputs'!B65="","",'Opportunity Inputs'!B65)</f>
         <v>0.8</v>
       </c>
     </row>
@@ -4812,7 +4812,7 @@
         <v>81</v>
       </c>
       <c r="C38" s="33" t="n">
-        <f aca="false">'Synergy Inputs'!B22</f>
+        <f aca="false">IF('Synergy Inputs'!B22="","",'Synergy Inputs'!B22)</f>
         <v>0.82</v>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
         <v>84</v>
       </c>
       <c r="C39" s="33" t="n">
-        <f aca="false">'Synergy Inputs'!B35</f>
+        <f aca="false">IF('Synergy Inputs'!B35="","",'Synergy Inputs'!B35)</f>
         <v>0.8</v>
       </c>
     </row>
@@ -4830,7 +4830,7 @@
         <v>455</v>
       </c>
       <c r="C41" s="1" t="str">
-        <f aca="false">IF(COUNTIF('Tier Assignment'!B5:B25,"Insufficient data")=0,"No sub-dimensions suppressed; full weight set applied; no responses excluded beyond validity screening","Sub-dimensions suppressed for insufficient data: "&amp;COUNTIF('Tier Assignment'!B5:B25,"Insufficient data")&amp;" (weights reallocated proportionally; see Tier Assignment)")</f>
+        <f aca="false">IF(COUNTIF('Composite Scoring'!$D$6:$D$25,0)=0,"No sub-dimensions suppressed; full weight set applied; no responses excluded beyond validity screening","Sub-dimensions suppressed for insufficient data: "&amp;COUNTIF('Composite Scoring'!$D$6:$D$25,0)&amp;" (weights reallocated proportionally; see Tier Assignment)")</f>
         <v>No sub-dimensions suppressed; full weight set applied; no responses excluded beyond validity screening</v>
       </c>
     </row>
@@ -5927,7 +5927,7 @@
         <v>379</v>
       </c>
       <c r="C87" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D11</f>
+        <f aca="false">IF('Engagement Metadata'!D11="","",'Engagement Metadata'!D11)</f>
         <v>Northwind Mutual</v>
       </c>
     </row>
@@ -5936,7 +5936,7 @@
         <v>380</v>
       </c>
       <c r="C88" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D12</f>
+        <f aca="false">IF('Engagement Metadata'!D12="","",'Engagement Metadata'!D12)</f>
         <v>Member Services</v>
       </c>
     </row>
@@ -5945,7 +5945,7 @@
         <v>14</v>
       </c>
       <c r="C89" s="35" t="n">
-        <f aca="false">'Engagement Metadata'!D13</f>
+        <f aca="false">IF('Engagement Metadata'!D13="","",'Engagement Metadata'!D13)</f>
         <v>60</v>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
         <v>491</v>
       </c>
       <c r="C90" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D14</f>
+        <f aca="false">IF('Engagement Metadata'!D14="","",'Engagement Metadata'!D14)</f>
         <v>K - Financial and Insurance Services</v>
       </c>
     </row>
@@ -5963,7 +5963,7 @@
         <v>17</v>
       </c>
       <c r="C91" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D15</f>
+        <f aca="false">IF('Engagement Metadata'!D15="","",'Engagement Metadata'!D15)</f>
         <v>Health insurance</v>
       </c>
     </row>
@@ -5972,7 +5972,7 @@
         <v>19</v>
       </c>
       <c r="C92" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D16</f>
+        <f aca="false">IF('Engagement Metadata'!D16="","",'Engagement Metadata'!D16)</f>
         <v>200–1,000 FTE</v>
       </c>
     </row>
@@ -5981,7 +5981,7 @@
         <v>21</v>
       </c>
       <c r="C93" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D17</f>
+        <f aca="false">IF('Engagement Metadata'!D17="","",'Engagement Metadata'!D17)</f>
         <v>Customer-facing service</v>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
         <v>492</v>
       </c>
       <c r="C94" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D18</f>
+        <f aca="false">IF('Engagement Metadata'!D18="","",'Engagement Metadata'!D18)</f>
         <v>Default</v>
       </c>
     </row>
@@ -5999,7 +5999,7 @@
         <v>25</v>
       </c>
       <c r="C95" s="38" t="n">
-        <f aca="false">'Engagement Metadata'!D19</f>
+        <f aca="false">IF('Engagement Metadata'!D19="","",'Engagement Metadata'!D19)</f>
         <v>46174</v>
       </c>
     </row>
@@ -6008,7 +6008,7 @@
         <v>26</v>
       </c>
       <c r="C96" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D20</f>
+        <f aca="false">IF('Engagement Metadata'!D20="","",'Engagement Metadata'!D20)</f>
         <v>M. (PerformanceVP)</v>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
         <v>493</v>
       </c>
       <c r="C97" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D21</f>
+        <f aca="false">IF('Engagement Metadata'!D21="","",'Engagement Metadata'!D21)</f>
         <v>PVP-2026-NWM-MS</v>
       </c>
     </row>
@@ -6054,7 +6054,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="str">
-        <f aca="false">'Engagement Metadata'!D12</f>
+        <f aca="false">IF('Engagement Metadata'!D12="","",'Engagement Metadata'!D12)</f>
         <v>Member Services</v>
       </c>
       <c r="B101" s="34" t="n">
@@ -7298,7 +7298,7 @@
         <v>46127</v>
       </c>
       <c r="E5" s="6" t="str">
-        <f aca="false">IFERROR(IF(B5="Insufficient data","n/a",IF(DATEDIF(D5,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D5,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C1",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B5="Insufficient data",B5=""),"n/a",IF(OR(NOT(ISNUMBER(D5)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D5,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D5,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C1",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F5" s="13" t="s">
@@ -7319,7 +7319,7 @@
         <v>46132</v>
       </c>
       <c r="E6" s="6" t="str">
-        <f aca="false">IFERROR(IF(B6="Insufficient data","n/a",IF(DATEDIF(D6,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D6,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C2",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B6="Insufficient data",B6=""),"n/a",IF(OR(NOT(ISNUMBER(D6)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D6,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D6,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C2",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F6" s="13"/>
@@ -7338,7 +7338,7 @@
         <v>46111</v>
       </c>
       <c r="E7" s="6" t="str">
-        <f aca="false">IFERROR(IF(B7="Insufficient data","n/a",IF(DATEDIF(D7,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D7,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C3",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B7="Insufficient data",B7=""),"n/a",IF(OR(NOT(ISNUMBER(D7)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D7,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D7,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C3",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F7" s="13" t="s">
@@ -7359,7 +7359,7 @@
         <v>46152</v>
       </c>
       <c r="E8" s="6" t="str">
-        <f aca="false">IFERROR(IF(B8="Insufficient data","n/a",IF(DATEDIF(D8,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C4",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D8,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C4",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B8="Insufficient data",B8=""),"n/a",IF(OR(NOT(ISNUMBER(D8)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D8,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C4",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D8,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C4",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F8" s="13" t="s">
@@ -7380,7 +7380,7 @@
         <v>46143</v>
       </c>
       <c r="E9" s="6" t="str">
-        <f aca="false">IFERROR(IF(B9="Insufficient data","n/a",IF(DATEDIF(D9,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C5",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D9,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C5",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B9="Insufficient data",B9=""),"n/a",IF(OR(NOT(ISNUMBER(D9)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D9,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("C5",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D9,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("C5",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F9" s="13"/>
@@ -7399,7 +7399,7 @@
         <v>46147</v>
       </c>
       <c r="E10" s="6" t="str">
-        <f aca="false">IFERROR(IF(B10="Insufficient data","n/a",IF(DATEDIF(D10,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("M1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D10,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("M1",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B10="Insufficient data",B10=""),"n/a",IF(OR(NOT(ISNUMBER(D10)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D10,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("M1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D10,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("M1",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F10" s="13"/>
@@ -7418,7 +7418,7 @@
         <v>46152</v>
       </c>
       <c r="E11" s="6" t="str">
-        <f aca="false">IFERROR(IF(B11="Insufficient data","n/a",IF(DATEDIF(D11,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("M2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D11,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("M2",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B11="Insufficient data",B11=""),"n/a",IF(OR(NOT(ISNUMBER(D11)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D11,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("M2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D11,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("M2",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F11" s="13"/>
@@ -7437,7 +7437,7 @@
         <v>46152</v>
       </c>
       <c r="E12" s="6" t="str">
-        <f aca="false">IFERROR(IF(B12="Insufficient data","n/a",IF(DATEDIF(D12,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("M3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D12,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("M3",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B12="Insufficient data",B12=""),"n/a",IF(OR(NOT(ISNUMBER(D12)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D12,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("M3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D12,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("M3",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F12" s="13"/>
@@ -7456,7 +7456,7 @@
         <v>46152</v>
       </c>
       <c r="E13" s="6" t="str">
-        <f aca="false">IFERROR(IF(B13="Insufficient data","n/a",IF(DATEDIF(D13,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("M4",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D13,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("M4",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B13="Insufficient data",B13=""),"n/a",IF(OR(NOT(ISNUMBER(D13)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D13,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("M4",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D13,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("M4",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F13" s="13"/>
@@ -7475,7 +7475,7 @@
         <v>46152</v>
       </c>
       <c r="E14" s="6" t="str">
-        <f aca="false">IFERROR(IF(B14="Insufficient data","n/a",IF(DATEDIF(D14,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("TW1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D14,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("TW1",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B14="Insufficient data",B14=""),"n/a",IF(OR(NOT(ISNUMBER(D14)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D14,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("TW1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D14,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("TW1",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F14" s="13"/>
@@ -7494,7 +7494,7 @@
         <v>46152</v>
       </c>
       <c r="E15" s="6" t="str">
-        <f aca="false">IFERROR(IF(B15="Insufficient data","n/a",IF(DATEDIF(D15,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("TW2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D15,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("TW2",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B15="Insufficient data",B15=""),"n/a",IF(OR(NOT(ISNUMBER(D15)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D15,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("TW2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D15,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("TW2",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F15" s="13"/>
@@ -7513,7 +7513,7 @@
         <v>46152</v>
       </c>
       <c r="E16" s="6" t="str">
-        <f aca="false">IFERROR(IF(B16="Insufficient data","n/a",IF(DATEDIF(D16,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("TW3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D16,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("TW3",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B16="Insufficient data",B16=""),"n/a",IF(OR(NOT(ISNUMBER(D16)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D16,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("TW3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D16,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("TW3",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F16" s="13" t="s">
@@ -7534,7 +7534,7 @@
         <v>46152</v>
       </c>
       <c r="E17" s="6" t="str">
-        <f aca="false">IFERROR(IF(B17="Insufficient data","n/a",IF(DATEDIF(D17,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D17,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O1",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B17="Insufficient data",B17=""),"n/a",IF(OR(NOT(ISNUMBER(D17)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D17,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D17,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O1",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F17" s="13" t="s">
@@ -7555,7 +7555,7 @@
         <v>46152</v>
       </c>
       <c r="E18" s="6" t="str">
-        <f aca="false">IFERROR(IF(B18="Insufficient data","n/a",IF(DATEDIF(D18,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D18,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O2",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B18="Insufficient data",B18=""),"n/a",IF(OR(NOT(ISNUMBER(D18)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D18,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D18,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O2",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F18" s="13" t="s">
@@ -7576,7 +7576,7 @@
         <v>46152</v>
       </c>
       <c r="E19" s="6" t="str">
-        <f aca="false">IFERROR(IF(B19="Insufficient data","n/a",IF(DATEDIF(D19,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D19,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O3",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B19="Insufficient data",B19=""),"n/a",IF(OR(NOT(ISNUMBER(D19)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D19,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D19,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O3",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F19" s="13" t="s">
@@ -7597,7 +7597,7 @@
         <v>46152</v>
       </c>
       <c r="E20" s="6" t="str">
-        <f aca="false">IFERROR(IF(B20="Insufficient data","n/a",IF(DATEDIF(D20,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O4",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D20,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O4",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B20="Insufficient data",B20=""),"n/a",IF(OR(NOT(ISNUMBER(D20)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D20,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O4",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D20,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O4",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F20" s="13"/>
@@ -7616,7 +7616,7 @@
         <v>46152</v>
       </c>
       <c r="E21" s="6" t="str">
-        <f aca="false">IFERROR(IF(B21="Insufficient data","n/a",IF(DATEDIF(D21,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O5",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D21,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O5",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B21="Insufficient data",B21=""),"n/a",IF(OR(NOT(ISNUMBER(D21)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D21,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("O5",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D21,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("O5",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F21" s="13" t="s">
@@ -7637,7 +7637,7 @@
         <v>46127</v>
       </c>
       <c r="E22" s="6" t="str">
-        <f aca="false">IFERROR(IF(B22="Insufficient data","n/a",IF(DATEDIF(D22,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("S1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D22,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("S1",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B22="Insufficient data",B22=""),"n/a",IF(OR(NOT(ISNUMBER(D22)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D22,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("S1",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D22,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("S1",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F22" s="13" t="s">
@@ -7658,7 +7658,7 @@
         <v>46152</v>
       </c>
       <c r="E23" s="6" t="str">
-        <f aca="false">IFERROR(IF(B23="Insufficient data","n/a",IF(DATEDIF(D23,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("S2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D23,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("S2",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B23="Insufficient data",B23=""),"n/a",IF(OR(NOT(ISNUMBER(D23)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D23,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("S2",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D23,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("S2",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F23" s="13" t="s">
@@ -7679,7 +7679,7 @@
         <v>46152</v>
       </c>
       <c r="E24" s="6" t="str">
-        <f aca="false">IFERROR(IF(B24="Insufficient data","n/a",IF(DATEDIF(D24,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("S3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D24,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("S3",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B24="Insufficient data",B24=""),"n/a",IF(OR(NOT(ISNUMBER(D24)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D24,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("S3",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D24,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("S3",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F24" s="13"/>
@@ -7698,7 +7698,7 @@
         <v>46157</v>
       </c>
       <c r="E25" s="6" t="str">
-        <f aca="false">IFERROR(IF(B25="Insufficient data","n/a",IF(DATEDIF(D25,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("DLP",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D25,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("DLP",Ref!$A$41:$A$61,0)),"Medium","Low"))),"-")</f>
+        <f aca="false">IFERROR(IF(OR(B25="Insufficient data",B25=""),"n/a",IF(OR(NOT(ISNUMBER(D25)),NOT(ISNUMBER('Engagement Metadata'!$D$19))),"Low",IF(DATEDIF(D25,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$B$41:$B$61,MATCH("DLP",Ref!$A$41:$A$61,0)),"High",IF(DATEDIF(D25,'Engagement Metadata'!$D$19,"m")&lt;=INDEX(Ref!$C$41:$C$61,MATCH("DLP",Ref!$A$41:$A$61,0)),"Medium","Low")))),"-")</f>
         <v>High</v>
       </c>
       <c r="F25" s="13" t="s">
@@ -7945,7 +7945,7 @@
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="19" t="n">
-        <f aca="false">IF('Tier Assignment'!$B$5="Tier 3",D13,IF('Tier Assignment'!$B$5="Insufficient data","",D12))</f>
+        <f aca="false">IF('Tier Assignment'!$B$5="Tier 3",IF(ISNUMBER(D13),D13,""),IF(OR('Tier Assignment'!$B$5="Insufficient data",'Tier Assignment'!$B$5=""),"",D12))</f>
         <v>76.1111111111111</v>
       </c>
     </row>
@@ -8513,7 +8513,7 @@
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="19" t="n">
-        <f aca="false">IF('Tier Assignment'!$B$9="Insufficient data","",IF('Tier Assignment'!$B$9="Tier 3",IF(ISNUMBER(B62),B62,""),IF(AND(ISNUMBER(B62),COUNT(B59:B61)&gt;0),AVERAGE(B59:B61)*0.6+B62*0.4,IF(COUNT(B59:B61)&gt;0,AVERAGE(B59:B61),IF(ISNUMBER(B62),B62,"")))))</f>
+        <f aca="false">IF(OR('Tier Assignment'!$B$9="Insufficient data",'Tier Assignment'!$B$9=""),"",IF('Tier Assignment'!$B$9="Tier 3",IF(ISNUMBER(B62),B62,""),IF(AND(ISNUMBER(B62),COUNT(B59:B61)&gt;0),AVERAGE(B59:B61)*0.6+B62*0.4,IF(COUNT(B59:B61)&gt;0,AVERAGE(B59:B61),IF(ISNUMBER(B62),B62,"")))))</f>
         <v>79</v>
       </c>
     </row>
@@ -8737,7 +8737,7 @@
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="19" t="n">
-        <f aca="false">IF('Tier Assignment'!$B$10="Insufficient data","",IF('Tier Assignment'!$B$10="Tier 3",D17,D5))</f>
+        <f aca="false">IF(OR('Tier Assignment'!$B$10="Insufficient data",'Tier Assignment'!$B$10=""),"",IF('Tier Assignment'!$B$10="Tier 3",D17,IF(ISNUMBER(D5),D5,"")))</f>
         <v>72</v>
       </c>
     </row>
@@ -9197,7 +9197,7 @@
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
       <c r="D8" s="16" t="n">
-        <f aca="false">IFERROR(0.4*D5+0.3*D6+0.3*D7,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(D5),ISNUMBER(D6),ISNUMBER(D7)),0.4*D5+0.3*D6+0.3*D7,"")</f>
         <v>62.3</v>
       </c>
     </row>
@@ -9352,7 +9352,7 @@
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="6" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D21),ABS(D21)&gt;15),"GAP - report separately","")</f>
+        <f aca="false">IF(ISNUMBER(D21),IF(ABS(D21)&gt;15,"GAP - report separately",""),"")</f>
         <v/>
       </c>
     </row>
@@ -9363,7 +9363,7 @@
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="19" t="n">
-        <f aca="false">IFERROR((D8+D20)/2,"")</f>
+        <f aca="false">IF(ISNUMBER(D21),IF(ABS(D21)&gt;15,D20,(D8+D20)/2),"")</f>
         <v>61.228125</v>
       </c>
     </row>
@@ -9412,7 +9412,7 @@
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="16" t="n">
-        <f aca="false">IFERROR(0.35*D26+0.4*D27+0.25*D28,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(D26),ISNUMBER(D27),ISNUMBER(D28)),0.35*D26+0.4*D27+0.25*D28,"")</f>
         <v>73.5</v>
       </c>
     </row>
@@ -9519,7 +9519,7 @@
       <c r="B39" s="10"/>
       <c r="C39" s="10"/>
       <c r="D39" s="6" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D38),ABS(D38)&gt;15),"GAP - report separately","")</f>
+        <f aca="false">IF(ISNUMBER(D38),IF(ABS(D38)&gt;15,"GAP - report separately",""),"")</f>
         <v/>
       </c>
     </row>
@@ -9530,7 +9530,7 @@
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="19" t="n">
-        <f aca="false">IFERROR((D29+D37)/2,"")</f>
+        <f aca="false">IF(ISNUMBER(D38),IF(ABS(D38)&gt;15,D37,(D29+D37)/2),"")</f>
         <v>69.25</v>
       </c>
     </row>
@@ -9559,7 +9559,7 @@
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="16" t="n">
-        <f aca="false">IFERROR(D43,"")</f>
+        <f aca="false">IF(ISNUMBER(D43),D43,"")</f>
         <v>60</v>
       </c>
     </row>
@@ -9678,7 +9678,7 @@
       <c r="B55" s="10"/>
       <c r="C55" s="10"/>
       <c r="D55" s="6" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D54),ABS(D54)&gt;15),"GAP - report separately","")</f>
+        <f aca="false">IF(ISNUMBER(D54),IF(ABS(D54)&gt;15,"GAP - report separately",""),"")</f>
         <v/>
       </c>
     </row>
@@ -9689,7 +9689,7 @@
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
       <c r="D56" s="19" t="n">
-        <f aca="false">IFERROR((D44+D53)/2,"")</f>
+        <f aca="false">IF(ISNUMBER(D54),IF(ABS(D54)&gt;15,D53,(D44+D53)/2),"")</f>
         <v>55.25</v>
       </c>
     </row>
@@ -9791,7 +9791,7 @@
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
       <c r="D67" s="19" t="n">
-        <f aca="false">IFERROR((D59+D66)/2,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(D59),ISNUMBER(D66)),(D59+D66)/2,"")</f>
         <v>47.5</v>
       </c>
     </row>
@@ -10015,7 +10015,7 @@
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="19" t="n">
-        <f aca="false">IFERROR(0.4*D5+0.35*D6+0.25*D7,"")</f>
+        <f aca="false">IF(AND(ISNUMBER(D5),ISNUMBER(D6),ISNUMBER(D7)),0.4*D5+0.35*D6+0.25*D7,"")</f>
         <v>85.75</v>
       </c>
     </row>
@@ -10188,7 +10188,7 @@
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="6" t="str">
-        <f aca="false">IF(AND(ISNUMBER(D24),ABS(D24)&gt;15),"GAP - diagnostic finding","")</f>
+        <f aca="false">IF(ISNUMBER(D24),IF(ABS(D24)&gt;15,"GAP - diagnostic finding",""),"")</f>
         <v>GAP - diagnostic finding</v>
       </c>
     </row>
@@ -10308,7 +10308,7 @@
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
       <c r="D37" s="6" t="str">
-        <f aca="false">IF(AND((B30-1)*25&lt;60,(B31-1)*25&lt;60,'Motivation Inputs'!$D$29&gt;75),"FALSE CONSENSUS - suppressed disagreement","")</f>
+        <f aca="false">IF(AND(ISNUMBER(B30),ISNUMBER(B31),ISNUMBER('Motivation Inputs'!$D$29)),IF(AND((B30-1)*25&lt;60,(B31-1)*25&lt;60,'Motivation Inputs'!$D$29&gt;75),"FALSE CONSENSUS - suppressed disagreement",""),"")</f>
         <v/>
       </c>
     </row>
@@ -11377,7 +11377,7 @@
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="6" t="str">
-        <f aca="false">IF(AND(ISNUMBER(C10),ABS(C10)&gt;15),"GAP - key finding","")</f>
+        <f aca="false">IF(ISNUMBER(C10),IF(ABS(C10)&gt;15,"GAP - key finding",""),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>